<commit_message>
fix: correct female-only study population metadata
</commit_message>
<xml_diff>
--- a/research_database/workbook/male_exercise_science_database_v3.0.0.xlsx
+++ b/research_database/workbook/male_exercise_science_database_v3.0.0.xlsx
@@ -1855,7 +1855,7 @@
     <t>Long-muscle-length partial calf raises increased gastrocnemius thickness more than short-length partials and, for some regions, full range of motion.</t>
   </si>
   <si>
-    <t>Female-only sample of 42 untrained young women; gastrocnemius-specific ultrasound outcomes cannot establish a male or whole-body rule. The mixed-sex contract flag is true because this cohort is not male-only, while the zero-male count and excluded applicability remain authoritative.</t>
+    <t>Female-only sample of 42 untrained young women; gastrocnemius-specific ultrasound outcomes cannot establish a male or whole-body rule. Because all 42 participants were women, the mixed-sex contract flag is false; the zero-male count and excluded applicability remain authoritative.</t>
   </si>
   <si>
     <t>Negative-control evidence row: retained for bibliography completeness but excluded from all male conclusions and application mappings.</t>
@@ -56889,7 +56889,7 @@
         <v>0</v>
       </c>
       <c r="N48" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O48" s="2" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
fix: preserve rule map ID epochs
</commit_message>
<xml_diff>
--- a/research_database/workbook/male_exercise_science_database_v3.0.0.xlsx
+++ b/research_database/workbook/male_exercise_science_database_v3.0.0.xlsx
@@ -7783,7 +7783,7 @@
     <t>3.0.0</t>
   </si>
   <si>
-    <t>research_library|evidence_conclusions|progression_rules|definitions_data_dictionary</t>
+    <t>research_library|evidence_conclusions|progression_rules|rule_exercise_map|definitions_data_dictionary</t>
   </si>
   <si>
     <t>stu_0043-stu_0048|con_0028-con_0031|rule_0001-rule_0019</t>
@@ -42380,10 +42380,10 @@
         <v>4260</v>
       </c>
       <c r="B755" s="2" t="s">
-        <v>1531</v>
+        <v>1396</v>
       </c>
       <c r="C755" s="2" t="s">
-        <v>1025</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="756" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42391,10 +42391,10 @@
         <v>4261</v>
       </c>
       <c r="B756" s="2" t="s">
-        <v>1531</v>
+        <v>1422</v>
       </c>
       <c r="C756" s="2" t="s">
-        <v>1055</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="757" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42402,10 +42402,10 @@
         <v>4262</v>
       </c>
       <c r="B757" s="2" t="s">
-        <v>1531</v>
+        <v>1428</v>
       </c>
       <c r="C757" s="2" t="s">
-        <v>1061</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="758" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42413,10 +42413,10 @@
         <v>4263</v>
       </c>
       <c r="B758" s="2" t="s">
-        <v>1531</v>
+        <v>1436</v>
       </c>
       <c r="C758" s="2" t="s">
-        <v>1067</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="759" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42424,10 +42424,10 @@
         <v>4264</v>
       </c>
       <c r="B759" s="2" t="s">
-        <v>1531</v>
+        <v>1445</v>
       </c>
       <c r="C759" s="2" t="s">
-        <v>1072</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="760" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42435,10 +42435,10 @@
         <v>4265</v>
       </c>
       <c r="B760" s="2" t="s">
-        <v>1531</v>
+        <v>1451</v>
       </c>
       <c r="C760" s="2" t="s">
-        <v>1078</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="761" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42446,10 +42446,10 @@
         <v>4266</v>
       </c>
       <c r="B761" s="2" t="s">
-        <v>1531</v>
+        <v>1458</v>
       </c>
       <c r="C761" s="2" t="s">
-        <v>1081</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="762" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42457,10 +42457,10 @@
         <v>4267</v>
       </c>
       <c r="B762" s="2" t="s">
-        <v>1531</v>
+        <v>1466</v>
       </c>
       <c r="C762" s="2" t="s">
-        <v>1090</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="763" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42468,10 +42468,10 @@
         <v>4268</v>
       </c>
       <c r="B763" s="2" t="s">
-        <v>1531</v>
+        <v>1474</v>
       </c>
       <c r="C763" s="2" t="s">
-        <v>1093</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="764" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42479,10 +42479,10 @@
         <v>4269</v>
       </c>
       <c r="B764" s="2" t="s">
-        <v>1531</v>
+        <v>1480</v>
       </c>
       <c r="C764" s="2" t="s">
-        <v>1100</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="765" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42490,10 +42490,10 @@
         <v>4270</v>
       </c>
       <c r="B765" s="2" t="s">
-        <v>1531</v>
+        <v>1488</v>
       </c>
       <c r="C765" s="2" t="s">
-        <v>1103</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="766" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42501,10 +42501,10 @@
         <v>4271</v>
       </c>
       <c r="B766" s="2" t="s">
-        <v>1531</v>
+        <v>1523</v>
       </c>
       <c r="C766" s="2" t="s">
-        <v>1109</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="767" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42515,7 +42515,7 @@
         <v>1531</v>
       </c>
       <c r="C767" s="2" t="s">
-        <v>1113</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="768" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42526,7 +42526,7 @@
         <v>1531</v>
       </c>
       <c r="C768" s="2" t="s">
-        <v>1116</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="769" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42537,7 +42537,7 @@
         <v>1531</v>
       </c>
       <c r="C769" s="2" t="s">
-        <v>1124</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="770" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42548,7 +42548,7 @@
         <v>1531</v>
       </c>
       <c r="C770" s="2" t="s">
-        <v>1127</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="771" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42559,7 +42559,7 @@
         <v>1531</v>
       </c>
       <c r="C771" s="2" t="s">
-        <v>1131</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="772" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42570,7 +42570,7 @@
         <v>1531</v>
       </c>
       <c r="C772" s="2" t="s">
-        <v>1134</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="773" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42581,7 +42581,7 @@
         <v>1531</v>
       </c>
       <c r="C773" s="2" t="s">
-        <v>1142</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="774" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42592,7 +42592,7 @@
         <v>1531</v>
       </c>
       <c r="C774" s="2" t="s">
-        <v>1145</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="775" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42603,7 +42603,7 @@
         <v>1531</v>
       </c>
       <c r="C775" s="2" t="s">
-        <v>1150</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="776" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42614,7 +42614,7 @@
         <v>1531</v>
       </c>
       <c r="C776" s="2" t="s">
-        <v>1155</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="777" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42625,7 +42625,7 @@
         <v>1531</v>
       </c>
       <c r="C777" s="2" t="s">
-        <v>1158</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="778" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42636,7 +42636,7 @@
         <v>1531</v>
       </c>
       <c r="C778" s="2" t="s">
-        <v>1163</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="779" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42647,7 +42647,7 @@
         <v>1531</v>
       </c>
       <c r="C779" s="2" t="s">
-        <v>1167</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="780" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42658,7 +42658,7 @@
         <v>1531</v>
       </c>
       <c r="C780" s="2" t="s">
-        <v>1177</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="781" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42669,7 +42669,7 @@
         <v>1531</v>
       </c>
       <c r="C781" s="2" t="s">
-        <v>1181</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="782" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42680,7 +42680,7 @@
         <v>1531</v>
       </c>
       <c r="C782" s="2" t="s">
-        <v>1185</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="783" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42691,7 +42691,7 @@
         <v>1531</v>
       </c>
       <c r="C783" s="2" t="s">
-        <v>1188</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="784" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42702,7 +42702,7 @@
         <v>1531</v>
       </c>
       <c r="C784" s="2" t="s">
-        <v>1193</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="785" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42713,7 +42713,7 @@
         <v>1531</v>
       </c>
       <c r="C785" s="2" t="s">
-        <v>1197</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="786" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42724,7 +42724,7 @@
         <v>1531</v>
       </c>
       <c r="C786" s="2" t="s">
-        <v>1205</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="787" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42735,7 +42735,7 @@
         <v>1531</v>
       </c>
       <c r="C787" s="2" t="s">
-        <v>1211</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="788" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42746,7 +42746,7 @@
         <v>1531</v>
       </c>
       <c r="C788" s="2" t="s">
-        <v>1216</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="789" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42757,7 +42757,7 @@
         <v>1531</v>
       </c>
       <c r="C789" s="2" t="s">
-        <v>1221</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="790" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42768,7 +42768,7 @@
         <v>1531</v>
       </c>
       <c r="C790" s="2" t="s">
-        <v>1226</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="791" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42779,7 +42779,7 @@
         <v>1531</v>
       </c>
       <c r="C791" s="2" t="s">
-        <v>1230</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="792" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42790,7 +42790,7 @@
         <v>1531</v>
       </c>
       <c r="C792" s="2" t="s">
-        <v>1233</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="793" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42801,7 +42801,7 @@
         <v>1531</v>
       </c>
       <c r="C793" s="2" t="s">
-        <v>1238</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="794" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42812,7 +42812,7 @@
         <v>1531</v>
       </c>
       <c r="C794" s="2" t="s">
-        <v>1243</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="795" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42823,7 +42823,7 @@
         <v>1531</v>
       </c>
       <c r="C795" s="2" t="s">
-        <v>1249</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="796" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42834,7 +42834,7 @@
         <v>1531</v>
       </c>
       <c r="C796" s="2" t="s">
-        <v>1252</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="797" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42845,7 +42845,7 @@
         <v>1531</v>
       </c>
       <c r="C797" s="2" t="s">
-        <v>1258</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="798" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42856,7 +42856,7 @@
         <v>1531</v>
       </c>
       <c r="C798" s="2" t="s">
-        <v>1262</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="799" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42867,7 +42867,7 @@
         <v>1531</v>
       </c>
       <c r="C799" s="2" t="s">
-        <v>1266</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="800" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42878,7 +42878,7 @@
         <v>1531</v>
       </c>
       <c r="C800" s="2" t="s">
-        <v>1271</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="801" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42889,7 +42889,7 @@
         <v>1531</v>
       </c>
       <c r="C801" s="2" t="s">
-        <v>1275</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="802" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42900,7 +42900,7 @@
         <v>1531</v>
       </c>
       <c r="C802" s="2" t="s">
-        <v>1278</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="803" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42911,7 +42911,7 @@
         <v>1531</v>
       </c>
       <c r="C803" s="2" t="s">
-        <v>1282</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="804" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42922,7 +42922,7 @@
         <v>1531</v>
       </c>
       <c r="C804" s="2" t="s">
-        <v>1287</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="805" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42933,7 +42933,7 @@
         <v>1531</v>
       </c>
       <c r="C805" s="2" t="s">
-        <v>1290</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="806" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42944,7 +42944,7 @@
         <v>1531</v>
       </c>
       <c r="C806" s="2" t="s">
-        <v>1294</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="807" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42955,7 +42955,7 @@
         <v>1531</v>
       </c>
       <c r="C807" s="2" t="s">
-        <v>1300</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="808" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42966,7 +42966,7 @@
         <v>1531</v>
       </c>
       <c r="C808" s="2" t="s">
-        <v>1304</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="809" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42977,7 +42977,7 @@
         <v>1531</v>
       </c>
       <c r="C809" s="2" t="s">
-        <v>1314</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="810" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42988,7 +42988,7 @@
         <v>1531</v>
       </c>
       <c r="C810" s="2" t="s">
-        <v>1319</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="811" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -42999,7 +42999,7 @@
         <v>1531</v>
       </c>
       <c r="C811" s="2" t="s">
-        <v>1324</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="812" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43010,7 +43010,7 @@
         <v>1531</v>
       </c>
       <c r="C812" s="2" t="s">
-        <v>1329</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="813" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43021,7 +43021,7 @@
         <v>1531</v>
       </c>
       <c r="C813" s="2" t="s">
-        <v>1336</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="814" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43032,7 +43032,7 @@
         <v>1531</v>
       </c>
       <c r="C814" s="2" t="s">
-        <v>984</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="815" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43043,7 +43043,7 @@
         <v>1531</v>
       </c>
       <c r="C815" s="2" t="s">
-        <v>989</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="816" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43051,10 +43051,10 @@
         <v>4321</v>
       </c>
       <c r="B816" s="2" t="s">
-        <v>1396</v>
+        <v>1531</v>
       </c>
       <c r="C816" s="2" t="s">
-        <v>1351</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="817" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43062,10 +43062,10 @@
         <v>4322</v>
       </c>
       <c r="B817" s="2" t="s">
-        <v>1422</v>
+        <v>1531</v>
       </c>
       <c r="C817" s="2" t="s">
-        <v>1351</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="818" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43073,10 +43073,10 @@
         <v>4323</v>
       </c>
       <c r="B818" s="2" t="s">
-        <v>1428</v>
+        <v>1531</v>
       </c>
       <c r="C818" s="2" t="s">
-        <v>1351</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="819" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43084,10 +43084,10 @@
         <v>4324</v>
       </c>
       <c r="B819" s="2" t="s">
-        <v>1436</v>
+        <v>1531</v>
       </c>
       <c r="C819" s="2" t="s">
-        <v>1351</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="820" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43095,10 +43095,10 @@
         <v>4325</v>
       </c>
       <c r="B820" s="2" t="s">
-        <v>1445</v>
+        <v>1531</v>
       </c>
       <c r="C820" s="2" t="s">
-        <v>1351</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="821" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43106,10 +43106,10 @@
         <v>4326</v>
       </c>
       <c r="B821" s="2" t="s">
-        <v>1451</v>
+        <v>1531</v>
       </c>
       <c r="C821" s="2" t="s">
-        <v>1351</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="822" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43117,10 +43117,10 @@
         <v>4327</v>
       </c>
       <c r="B822" s="2" t="s">
-        <v>1458</v>
+        <v>1531</v>
       </c>
       <c r="C822" s="2" t="s">
-        <v>1351</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="823" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43128,10 +43128,10 @@
         <v>4328</v>
       </c>
       <c r="B823" s="2" t="s">
-        <v>1466</v>
+        <v>1531</v>
       </c>
       <c r="C823" s="2" t="s">
-        <v>1351</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="824" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43139,10 +43139,10 @@
         <v>4329</v>
       </c>
       <c r="B824" s="2" t="s">
-        <v>1474</v>
+        <v>1531</v>
       </c>
       <c r="C824" s="2" t="s">
-        <v>1351</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="825" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43150,10 +43150,10 @@
         <v>4330</v>
       </c>
       <c r="B825" s="2" t="s">
-        <v>1480</v>
+        <v>1531</v>
       </c>
       <c r="C825" s="2" t="s">
-        <v>1351</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="826" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43161,10 +43161,10 @@
         <v>4331</v>
       </c>
       <c r="B826" s="2" t="s">
-        <v>1488</v>
+        <v>1531</v>
       </c>
       <c r="C826" s="2" t="s">
-        <v>1351</v>
+        <v>984</v>
       </c>
     </row>
     <row r="827" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -43172,10 +43172,10 @@
         <v>4332</v>
       </c>
       <c r="B827" s="2" t="s">
-        <v>1523</v>
+        <v>1531</v>
       </c>
       <c r="C827" s="2" t="s">
-        <v>1351</v>
+        <v>989</v>
       </c>
     </row>
     <row r="828" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix Strong exercise identity aliases
</commit_message>
<xml_diff>
--- a/research_database/workbook/male_exercise_science_database_v3.0.0.xlsx
+++ b/research_database/workbook/male_exercise_science_database_v3.0.0.xlsx
@@ -3112,7 +3112,7 @@
     <t>Barbell Bench Press</t>
   </si>
   <si>
-    <t>bench press</t>
+    <t>bench press|bench press (barbell)</t>
   </si>
   <si>
     <t>horizontal_push</t>
@@ -3238,7 +3238,7 @@
     <t>Incline Dumbbell Press</t>
   </si>
   <si>
-    <t>incline db press</t>
+    <t>incline db press|incline bench press (dumbbell)</t>
   </si>
   <si>
     <t>dumbbells_and_incline_bench</t>
@@ -3346,7 +3346,7 @@
     <t>Cable Lateral Raise</t>
   </si>
   <si>
-    <t>one arm cable lateral raise</t>
+    <t>one arm cable lateral raise|lateral raise (cable)</t>
   </si>
   <si>
     <t>shoulder_abduction</t>
@@ -3418,7 +3418,7 @@
     <t>Lat Pulldown</t>
   </si>
   <si>
-    <t>cable pulldown</t>
+    <t>cable pulldown|lat pulldown double pulley</t>
   </si>
   <si>
     <t>cable_machine</t>
@@ -3616,7 +3616,7 @@
     <t>Leg Extension</t>
   </si>
   <si>
-    <t>knee extension machine</t>
+    <t>knee extension machine|leg extension (machine)|leg extension (heavy)</t>
   </si>
   <si>
     <t>knee_extension</t>
@@ -3715,7 +3715,7 @@
     <t>Seated Leg Curl</t>
   </si>
   <si>
-    <t>seated hamstring curl</t>
+    <t>seated hamstring curl|seated leg curl (machine)</t>
   </si>
   <si>
     <t>knee_flexion</t>
@@ -3727,7 +3727,7 @@
     <t>Lying Leg Curl</t>
   </si>
   <si>
-    <t>prone hamstring curl</t>
+    <t>prone hamstring curl|lying leg curl (machine)</t>
   </si>
   <si>
     <t>ex_nordic_curl</t>
@@ -3793,7 +3793,7 @@
     <t>Standing Calf Raise</t>
   </si>
   <si>
-    <t>straight knee calf raise</t>
+    <t>straight knee calf raise|standing calf raise (machine)</t>
   </si>
   <si>
     <t>plantar_flexion</t>
@@ -3823,7 +3823,7 @@
     <t>Leg Press Calf Raise</t>
   </si>
   <si>
-    <t>calf press</t>
+    <t>calf press|calf press on seated leg press</t>
   </si>
   <si>
     <t>leg_press</t>
@@ -3835,7 +3835,7 @@
     <t>Incline Dumbbell Curl</t>
   </si>
   <si>
-    <t>incline curl</t>
+    <t>incline curl|incline curl (dumbbell)</t>
   </si>
   <si>
     <t>elbow_flexion</t>
@@ -3862,7 +3862,7 @@
     <t>Cable Curl</t>
   </si>
   <si>
-    <t>standing cable curl</t>
+    <t>standing cable curl|bicep curl (cable)|bicep curls light (cable)</t>
   </si>
   <si>
     <t>ex_hammer_curl</t>
@@ -3883,7 +3883,7 @@
     <t>Cable Triceps Pushdown</t>
   </si>
   <si>
-    <t>triceps pressdown</t>
+    <t>triceps pressdown|triceps pushdown (cable - straight bar)|tricep pushdown - dongles</t>
   </si>
   <si>
     <t>elbow_extension</t>
@@ -4009,7 +4009,7 @@
     <t>Ab Wheel Rollout</t>
   </si>
   <si>
-    <t>ab rollout</t>
+    <t>ab rollout|ab wheel</t>
   </si>
   <si>
     <t>anti_extension</t>
@@ -4054,7 +4054,7 @@
     <t>Neck Flexion</t>
   </si>
   <si>
-    <t>weighted neck curl</t>
+    <t>weighted neck curl|neck curls (front)</t>
   </si>
   <si>
     <t>neck_flexion</t>
@@ -4072,7 +4072,7 @@
     <t>Neck Extension</t>
   </si>
   <si>
-    <t>neck harness extension</t>
+    <t>neck harness extension|neck curls (back)</t>
   </si>
   <si>
     <t>neck_extension</t>

</xml_diff>